<commit_message>
ui changes, changed way it works
</commit_message>
<xml_diff>
--- a/finance_db.xlsx
+++ b/finance_db.xlsx
@@ -10,7 +10,10 @@
     <sheet name="Budget" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Vendors" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Projects" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cheque Distribution" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Divisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Districts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Entries" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Entry Gadgets" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,10 +456,10 @@
         <v>1000000</v>
       </c>
       <c r="B2" t="n">
-        <v>350000</v>
+        <v>23700</v>
       </c>
       <c r="C2" t="n">
-        <v>650000</v>
+        <v>976300</v>
       </c>
     </row>
   </sheetData>
@@ -470,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,15 +484,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Vendor Code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Total Billed</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Total Paid</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Balance Due</t>
         </is>
@@ -501,14 +509,19 @@
           <t>ABC Pvt Ltd</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>V001</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>300000</v>
       </c>
-      <c r="C2" t="n">
-        <v>250000</v>
-      </c>
       <c r="D2" t="n">
-        <v>50000</v>
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>300000</v>
       </c>
     </row>
     <row r="3">
@@ -517,14 +530,40 @@
           <t>XYZ Infra</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>V002</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>200000</v>
       </c>
-      <c r="C3" t="n">
-        <v>100000</v>
-      </c>
       <c r="D3" t="n">
-        <v>100000</v>
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sg pvt.ltd</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>V003</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>23700</v>
+      </c>
+      <c r="D4" t="n">
+        <v>23700</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -538,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,55 +591,29 @@
           <t>Project Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Vendor Assigned</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Total Project Cost</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Road Work</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>ABC Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>300000</v>
+          <t>Bandhara</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Drain Work</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>XYZ Infra</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>200000</v>
+          <t>wall construction</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -614,134 +627,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Vendor Name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Cheque Amount</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Division Name</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>ABC Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Road Work</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>200000</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Issued</t>
+          <t>Amravati</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-12 02:22:41</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ABC Pvt Ltd</t>
-        </is>
+          <t>Sambhainagar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>District Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Akola</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Jalna</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Entry ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Vendor Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Vendor Code</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Check No</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Gross Amount</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Gadget Count</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-03-15 18:14:54</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>sg pvt.ltd</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>V003</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>23700</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Entry ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Gadget No</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Gadget Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Project Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Division</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>District</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Taluka</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Project Details</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Total Amount</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Security Deposit</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>GST</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Tax</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Vima</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Kamgar Kalyan</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Total Deduction</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Gross Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E0001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>G001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bandhara</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Amravati</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Akola</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Akot</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>bla bla</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="J2" t="n">
+        <v>300</v>
+      </c>
+      <c r="K2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L2" t="n">
+        <v>100</v>
+      </c>
+      <c r="M2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N2" t="n">
+        <v>100</v>
+      </c>
+      <c r="O2" t="n">
+        <v>700</v>
+      </c>
+      <c r="P2" t="n">
+        <v>14300</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E0001</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Road Work</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>50000</v>
+          <t>G002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>wall construction</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Issued</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-03-12 02:23:28</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>XYZ Infra</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Road Work</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Issued</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-03-12 02:23:52</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>XYZ Infra</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Drain Work</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Issued</t>
-        </is>
+          <t>Sambhainagar</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Jalna</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Jalna</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>bla bla</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J3" t="n">
+        <v>200</v>
+      </c>
+      <c r="K3" t="n">
+        <v>100</v>
+      </c>
+      <c r="L3" t="n">
+        <v>100</v>
+      </c>
+      <c r="M3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N3" t="n">
+        <v>100</v>
+      </c>
+      <c r="O3" t="n">
+        <v>600</v>
+      </c>
+      <c r="P3" t="n">
+        <v>9400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>